<commit_message>
Harden SUMO input cleaning and audit contract
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/validation/sumo_input_do_v3_20260919/outputs/dqr_forcing/DQR_DO_ORP_export_audit.xlsx
+++ b/Project 1 Data Quality Assessment/validation/sumo_input_do_v3_20260919/outputs/dqr_forcing/DQR_DO_ORP_export_audit.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels" sheetId="1" r:id="Ra9423b6a92b7434d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Months" sheetId="2" r:id="Rbbc71a881cb548ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Windows" sheetId="3" r:id="R3146c8d0773a4cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessCoverage" sheetId="4" r:id="R14e58ac48fab48a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract" sheetId="5" r:id="R542f2d34bba04354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels" sheetId="1" r:id="Ra1adf1079f014e2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Months" sheetId="2" r:id="R91cb7d0389454af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Windows" sheetId="3" r:id="R25eeac0e481a40ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessCoverage" sheetId="4" r:id="R257bf0ecdd004d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract" sheetId="5" r:id="R41d75f041afe4e97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2470,16 +2470,16 @@
         <x:v>46112</x:v>
       </x:c>
       <x:c r="C22" s="14" t="n">
-        <x:v>46121.62847222222</x:v>
+        <x:v>46151.711805555555</x:v>
       </x:c>
       <x:c r="D22" s="13" t="n">
-        <x:v>9.6284722222</x:v>
+        <x:v>39.7118055556</x:v>
       </x:c>
       <x:c r="E22" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F22" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>25.7118055556</x:v>
       </x:c>
       <x:c r="G22" s="15" t="b">
         <x:v>0</x:v>
@@ -2490,22 +2490,22 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B23" s="14" t="n">
-        <x:v>46121.631944444445</x:v>
+        <x:v>46151.81597222222</x:v>
       </x:c>
       <x:c r="C23" s="14" t="n">
-        <x:v>46121.729166666664</x:v>
+        <x:v>46202.510416666664</x:v>
       </x:c>
       <x:c r="D23" s="13" t="n">
-        <x:v>0.0972222222</x:v>
+        <x:v>50.6944444444</x:v>
       </x:c>
       <x:c r="E23" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F23" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>36.6944444444</x:v>
       </x:c>
       <x:c r="G23" s="15" t="b">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
@@ -2513,19 +2513,19 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B24" s="14" t="n">
-        <x:v>46121.75</x:v>
+        <x:v>46202.631944444445</x:v>
       </x:c>
       <x:c r="C24" s="14" t="n">
-        <x:v>46151.711805555555</x:v>
+        <x:v>46202.68402777778</x:v>
       </x:c>
       <x:c r="D24" s="13" t="n">
-        <x:v>29.9618055556</x:v>
+        <x:v>0.0520833333</x:v>
       </x:c>
       <x:c r="E24" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F24" s="13" t="n">
-        <x:v>15.9618055556</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G24" s="15" t="b">
         <x:v>0</x:v>
@@ -2536,19 +2536,19 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B25" s="14" t="n">
-        <x:v>46151.81597222222</x:v>
+        <x:v>46202.979166666664</x:v>
       </x:c>
       <x:c r="C25" s="14" t="n">
-        <x:v>46180.552083333336</x:v>
+        <x:v>46203.45138888889</x:v>
       </x:c>
       <x:c r="D25" s="13" t="n">
-        <x:v>28.7361111111</x:v>
+        <x:v>0.4722222222</x:v>
       </x:c>
       <x:c r="E25" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F25" s="13" t="n">
-        <x:v>14.7361111111</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G25" s="15" t="b">
         <x:v>0</x:v>
@@ -2559,19 +2559,19 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B26" s="14" t="n">
-        <x:v>46180.555555555555</x:v>
+        <x:v>46203.461805555555</x:v>
       </x:c>
       <x:c r="C26" s="14" t="n">
-        <x:v>46195.663194444445</x:v>
+        <x:v>46203.475694444445</x:v>
       </x:c>
       <x:c r="D26" s="13" t="n">
-        <x:v>15.1076388889</x:v>
+        <x:v>0.0138888889</x:v>
       </x:c>
       <x:c r="E26" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F26" s="13" t="n">
-        <x:v>1.1076388889</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G26" s="15" t="b">
         <x:v>0</x:v>
@@ -2582,13 +2582,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B27" s="14" t="n">
-        <x:v>46195.694444444445</x:v>
+        <x:v>46203.57986111111</x:v>
       </x:c>
       <x:c r="C27" s="14" t="n">
-        <x:v>46196.55902777778</x:v>
+        <x:v>46203.583333333336</x:v>
       </x:c>
       <x:c r="D27" s="13" t="n">
-        <x:v>0.8645833333</x:v>
+        <x:v>0.0034722222</x:v>
       </x:c>
       <x:c r="E27" s="13" t="n">
         <x:v>14</x:v>
@@ -2605,13 +2605,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B28" s="14" t="n">
-        <x:v>46196.569444444445</x:v>
+        <x:v>46203.60763888889</x:v>
       </x:c>
       <x:c r="C28" s="14" t="n">
-        <x:v>46199.59722222222</x:v>
+        <x:v>46203.62152777778</x:v>
       </x:c>
       <x:c r="D28" s="13" t="n">
-        <x:v>3.0277777778</x:v>
+        <x:v>0.0138888889</x:v>
       </x:c>
       <x:c r="E28" s="13" t="n">
         <x:v>14</x:v>
@@ -2628,13 +2628,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B29" s="14" t="n">
-        <x:v>46199.600694444445</x:v>
+        <x:v>46203.631944444445</x:v>
       </x:c>
       <x:c r="C29" s="14" t="n">
-        <x:v>46202.510416666664</x:v>
+        <x:v>46203.64236111111</x:v>
       </x:c>
       <x:c r="D29" s="13" t="n">
-        <x:v>2.9097222222</x:v>
+        <x:v>0.0104166667</x:v>
       </x:c>
       <x:c r="E29" s="13" t="n">
         <x:v>14</x:v>
@@ -2651,13 +2651,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B30" s="14" t="n">
-        <x:v>46202.631944444445</x:v>
+        <x:v>46203.645833333336</x:v>
       </x:c>
       <x:c r="C30" s="14" t="n">
-        <x:v>46202.6875</x:v>
+        <x:v>46203.649305555555</x:v>
       </x:c>
       <x:c r="D30" s="13" t="n">
-        <x:v>0.0555555556</x:v>
+        <x:v>0.0034722222</x:v>
       </x:c>
       <x:c r="E30" s="13" t="n">
         <x:v>14</x:v>
@@ -2674,13 +2674,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B31" s="14" t="n">
-        <x:v>46202.979166666664</x:v>
+        <x:v>46203.65277777778</x:v>
       </x:c>
       <x:c r="C31" s="14" t="n">
-        <x:v>46203.45138888889</x:v>
+        <x:v>46203.663194444445</x:v>
       </x:c>
       <x:c r="D31" s="13" t="n">
-        <x:v>0.4722222222</x:v>
+        <x:v>0.0104166667</x:v>
       </x:c>
       <x:c r="E31" s="13" t="n">
         <x:v>14</x:v>
@@ -2697,13 +2697,13 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B32" s="14" t="n">
-        <x:v>46203.461805555555</x:v>
+        <x:v>46203.67013888889</x:v>
       </x:c>
       <x:c r="C32" s="14" t="n">
-        <x:v>46203.475694444445</x:v>
+        <x:v>46209.59027777778</x:v>
       </x:c>
       <x:c r="D32" s="13" t="n">
-        <x:v>0.0138888889</x:v>
+        <x:v>5.9201388889</x:v>
       </x:c>
       <x:c r="E32" s="13" t="n">
         <x:v>14</x:v>
@@ -2720,1516 +2720,21 @@
         <x:v>Eight DO + 12 process inputs (units pending)</x:v>
       </x:c>
       <x:c r="B33" s="14" t="n">
-        <x:v>46203.57986111111</x:v>
+        <x:v>46209.59722222222</x:v>
       </x:c>
       <x:c r="C33" s="14" t="n">
-        <x:v>46203.583333333336</x:v>
+        <x:v>46233.90625</x:v>
       </x:c>
       <x:c r="D33" s="13" t="n">
-        <x:v>0.0034722222</x:v>
+        <x:v>24.3090277778</x:v>
       </x:c>
       <x:c r="E33" s="13" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F33" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>10.3090277778</x:v>
       </x:c>
       <x:c r="G33" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="36" customHeight="1">
-      <x:c r="A34" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B34" s="14" t="n">
-        <x:v>46203.60763888889</x:v>
-      </x:c>
-      <x:c r="C34" s="14" t="n">
-        <x:v>46203.62152777778</x:v>
-      </x:c>
-      <x:c r="D34" s="13" t="n">
-        <x:v>0.0138888889</x:v>
-      </x:c>
-      <x:c r="E34" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F34" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G34" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="36" customHeight="1">
-      <x:c r="A35" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B35" s="14" t="n">
-        <x:v>46203.631944444445</x:v>
-      </x:c>
-      <x:c r="C35" s="14" t="n">
-        <x:v>46203.64236111111</x:v>
-      </x:c>
-      <x:c r="D35" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E35" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F35" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G35" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="36" customHeight="1">
-      <x:c r="A36" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B36" s="14" t="n">
-        <x:v>46203.645833333336</x:v>
-      </x:c>
-      <x:c r="C36" s="14" t="n">
-        <x:v>46203.649305555555</x:v>
-      </x:c>
-      <x:c r="D36" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E36" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F36" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G36" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="36" customHeight="1">
-      <x:c r="A37" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B37" s="14" t="n">
-        <x:v>46203.65277777778</x:v>
-      </x:c>
-      <x:c r="C37" s="14" t="n">
-        <x:v>46203.663194444445</x:v>
-      </x:c>
-      <x:c r="D37" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E37" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F37" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G37" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="36" customHeight="1">
-      <x:c r="A38" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B38" s="14" t="n">
-        <x:v>46203.67013888889</x:v>
-      </x:c>
-      <x:c r="C38" s="14" t="n">
-        <x:v>46209.59027777778</x:v>
-      </x:c>
-      <x:c r="D38" s="13" t="n">
-        <x:v>5.9201388889</x:v>
-      </x:c>
-      <x:c r="E38" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F38" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G38" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="36" customHeight="1">
-      <x:c r="A39" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B39" s="14" t="n">
-        <x:v>46209.59722222222</x:v>
-      </x:c>
-      <x:c r="C39" s="14" t="n">
-        <x:v>46209.635416666664</x:v>
-      </x:c>
-      <x:c r="D39" s="13" t="n">
-        <x:v>0.0381944444</x:v>
-      </x:c>
-      <x:c r="E39" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F39" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G39" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="36" customHeight="1">
-      <x:c r="A40" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B40" s="14" t="n">
-        <x:v>46209.64236111111</x:v>
-      </x:c>
-      <x:c r="C40" s="14" t="n">
-        <x:v>46210.211805555555</x:v>
-      </x:c>
-      <x:c r="D40" s="13" t="n">
-        <x:v>0.5694444444</x:v>
-      </x:c>
-      <x:c r="E40" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F40" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G40" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="36" customHeight="1">
-      <x:c r="A41" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B41" s="14" t="n">
-        <x:v>46210.21527777778</x:v>
-      </x:c>
-      <x:c r="C41" s="14" t="n">
-        <x:v>46210.225694444445</x:v>
-      </x:c>
-      <x:c r="D41" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E41" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F41" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G41" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="36" customHeight="1">
-      <x:c r="A42" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B42" s="14" t="n">
-        <x:v>46210.23263888889</x:v>
-      </x:c>
-      <x:c r="C42" s="14" t="n">
-        <x:v>46210.25</x:v>
-      </x:c>
-      <x:c r="D42" s="13" t="n">
-        <x:v>0.0173611111</x:v>
-      </x:c>
-      <x:c r="E42" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F42" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G42" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="36" customHeight="1">
-      <x:c r="A43" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B43" s="14" t="n">
-        <x:v>46210.25347222222</x:v>
-      </x:c>
-      <x:c r="C43" s="14" t="n">
-        <x:v>46210.274305555555</x:v>
-      </x:c>
-      <x:c r="D43" s="13" t="n">
-        <x:v>0.0208333333</x:v>
-      </x:c>
-      <x:c r="E43" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F43" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G43" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="36" customHeight="1">
-      <x:c r="A44" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B44" s="14" t="n">
-        <x:v>46210.27777777778</x:v>
-      </x:c>
-      <x:c r="C44" s="14" t="n">
-        <x:v>46210.336805555555</x:v>
-      </x:c>
-      <x:c r="D44" s="13" t="n">
-        <x:v>0.0590277778</x:v>
-      </x:c>
-      <x:c r="E44" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F44" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G44" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="36" customHeight="1">
-      <x:c r="A45" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B45" s="14" t="n">
-        <x:v>46210.34027777778</x:v>
-      </x:c>
-      <x:c r="C45" s="14" t="n">
-        <x:v>46210.34375</x:v>
-      </x:c>
-      <x:c r="D45" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E45" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F45" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G45" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="36" customHeight="1">
-      <x:c r="A46" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B46" s="14" t="n">
-        <x:v>46210.350694444445</x:v>
-      </x:c>
-      <x:c r="C46" s="14" t="n">
-        <x:v>46210.37152777778</x:v>
-      </x:c>
-      <x:c r="D46" s="13" t="n">
-        <x:v>0.0208333333</x:v>
-      </x:c>
-      <x:c r="E46" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F46" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G46" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="36" customHeight="1">
-      <x:c r="A47" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B47" s="14" t="n">
-        <x:v>46210.38888888889</x:v>
-      </x:c>
-      <x:c r="C47" s="14" t="n">
-        <x:v>46210.40625</x:v>
-      </x:c>
-      <x:c r="D47" s="13" t="n">
-        <x:v>0.0173611111</x:v>
-      </x:c>
-      <x:c r="E47" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F47" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G47" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="36" customHeight="1">
-      <x:c r="A48" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B48" s="14" t="n">
-        <x:v>46210.413194444445</x:v>
-      </x:c>
-      <x:c r="C48" s="14" t="n">
-        <x:v>46210.42013888889</x:v>
-      </x:c>
-      <x:c r="D48" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E48" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F48" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G48" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="36" customHeight="1">
-      <x:c r="A49" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B49" s="14" t="n">
-        <x:v>46210.427083333336</x:v>
-      </x:c>
-      <x:c r="C49" s="14" t="n">
-        <x:v>46210.44097222222</x:v>
-      </x:c>
-      <x:c r="D49" s="13" t="n">
-        <x:v>0.0138888889</x:v>
-      </x:c>
-      <x:c r="E49" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F49" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G49" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="36" customHeight="1">
-      <x:c r="A50" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B50" s="14" t="n">
-        <x:v>46210.447916666664</x:v>
-      </x:c>
-      <x:c r="C50" s="14" t="n">
-        <x:v>46210.458333333336</x:v>
-      </x:c>
-      <x:c r="D50" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E50" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F50" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G50" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="36" customHeight="1">
-      <x:c r="A51" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B51" s="14" t="n">
-        <x:v>46210.46527777778</x:v>
-      </x:c>
-      <x:c r="C51" s="14" t="n">
-        <x:v>46210.475694444445</x:v>
-      </x:c>
-      <x:c r="D51" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E51" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F51" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G51" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="36" customHeight="1">
-      <x:c r="A52" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B52" s="14" t="n">
-        <x:v>46210.48263888889</x:v>
-      </x:c>
-      <x:c r="C52" s="14" t="n">
-        <x:v>46211.625</x:v>
-      </x:c>
-      <x:c r="D52" s="13" t="n">
-        <x:v>1.1423611111</x:v>
-      </x:c>
-      <x:c r="E52" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F52" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G52" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="36" customHeight="1">
-      <x:c r="A53" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B53" s="14" t="n">
-        <x:v>46211.62847222222</x:v>
-      </x:c>
-      <x:c r="C53" s="14" t="n">
-        <x:v>46214.958333333336</x:v>
-      </x:c>
-      <x:c r="D53" s="13" t="n">
-        <x:v>3.3298611111</x:v>
-      </x:c>
-      <x:c r="E53" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F53" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G53" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="36" customHeight="1">
-      <x:c r="A54" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B54" s="14" t="n">
-        <x:v>46214.961805555555</x:v>
-      </x:c>
-      <x:c r="C54" s="14" t="n">
-        <x:v>46214.96875</x:v>
-      </x:c>
-      <x:c r="D54" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E54" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F54" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G54" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="36" customHeight="1">
-      <x:c r="A55" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B55" s="14" t="n">
-        <x:v>46214.97222222222</x:v>
-      </x:c>
-      <x:c r="C55" s="14" t="n">
-        <x:v>46215.07986111111</x:v>
-      </x:c>
-      <x:c r="D55" s="13" t="n">
-        <x:v>0.1076388889</x:v>
-      </x:c>
-      <x:c r="E55" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F55" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G55" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="36" customHeight="1">
-      <x:c r="A56" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B56" s="14" t="n">
-        <x:v>46215.083333333336</x:v>
-      </x:c>
-      <x:c r="C56" s="14" t="n">
-        <x:v>46215.086805555555</x:v>
-      </x:c>
-      <x:c r="D56" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E56" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F56" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G56" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="36" customHeight="1">
-      <x:c r="A57" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B57" s="14" t="n">
-        <x:v>46215.09027777778</x:v>
-      </x:c>
-      <x:c r="C57" s="14" t="n">
-        <x:v>46215.09375</x:v>
-      </x:c>
-      <x:c r="D57" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E57" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F57" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G57" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="36" customHeight="1">
-      <x:c r="A58" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B58" s="14" t="n">
-        <x:v>46215.100694444445</x:v>
-      </x:c>
-      <x:c r="C58" s="14" t="n">
-        <x:v>46215.49652777778</x:v>
-      </x:c>
-      <x:c r="D58" s="13" t="n">
-        <x:v>0.3958333333</x:v>
-      </x:c>
-      <x:c r="E58" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F58" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G58" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="36" customHeight="1">
-      <x:c r="A59" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B59" s="14" t="n">
-        <x:v>46215.510416666664</x:v>
-      </x:c>
-      <x:c r="C59" s="14" t="n">
-        <x:v>46218.54861111111</x:v>
-      </x:c>
-      <x:c r="D59" s="13" t="n">
-        <x:v>3.0381944444</x:v>
-      </x:c>
-      <x:c r="E59" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F59" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G59" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="36" customHeight="1">
-      <x:c r="A60" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B60" s="14" t="n">
-        <x:v>46218.552083333336</x:v>
-      </x:c>
-      <x:c r="C60" s="14" t="n">
-        <x:v>46224.93402777778</x:v>
-      </x:c>
-      <x:c r="D60" s="13" t="n">
-        <x:v>6.3819444444</x:v>
-      </x:c>
-      <x:c r="E60" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F60" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G60" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="36" customHeight="1">
-      <x:c r="A61" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B61" s="14" t="n">
-        <x:v>46224.94097222222</x:v>
-      </x:c>
-      <x:c r="C61" s="14" t="n">
-        <x:v>46224.95138888889</x:v>
-      </x:c>
-      <x:c r="D61" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E61" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F61" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G61" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="36" customHeight="1">
-      <x:c r="A62" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B62" s="14" t="n">
-        <x:v>46224.96527777778</x:v>
-      </x:c>
-      <x:c r="C62" s="14" t="n">
-        <x:v>46228.13888888889</x:v>
-      </x:c>
-      <x:c r="D62" s="13" t="n">
-        <x:v>3.1736111111</x:v>
-      </x:c>
-      <x:c r="E62" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F62" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G62" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="36" customHeight="1">
-      <x:c r="A63" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B63" s="14" t="n">
-        <x:v>46228.149305555555</x:v>
-      </x:c>
-      <x:c r="C63" s="14" t="n">
-        <x:v>46229.135416666664</x:v>
-      </x:c>
-      <x:c r="D63" s="13" t="n">
-        <x:v>0.9861111111</x:v>
-      </x:c>
-      <x:c r="E63" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F63" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G63" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="36" customHeight="1">
-      <x:c r="A64" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B64" s="14" t="n">
-        <x:v>46229.13888888889</x:v>
-      </x:c>
-      <x:c r="C64" s="14" t="n">
-        <x:v>46229.14236111111</x:v>
-      </x:c>
-      <x:c r="D64" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E64" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F64" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G64" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="36" customHeight="1">
-      <x:c r="A65" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B65" s="14" t="n">
-        <x:v>46229.15625</x:v>
-      </x:c>
-      <x:c r="C65" s="14" t="n">
-        <x:v>46229.239583333336</x:v>
-      </x:c>
-      <x:c r="D65" s="13" t="n">
-        <x:v>0.0833333333</x:v>
-      </x:c>
-      <x:c r="E65" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F65" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G65" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="36" customHeight="1">
-      <x:c r="A66" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B66" s="14" t="n">
-        <x:v>46229.24652777778</x:v>
-      </x:c>
-      <x:c r="C66" s="14" t="n">
-        <x:v>46229.25347222222</x:v>
-      </x:c>
-      <x:c r="D66" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E66" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F66" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G66" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="36" customHeight="1">
-      <x:c r="A67" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B67" s="14" t="n">
-        <x:v>46229.256944444445</x:v>
-      </x:c>
-      <x:c r="C67" s="14" t="n">
-        <x:v>46229.26388888889</x:v>
-      </x:c>
-      <x:c r="D67" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E67" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F67" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G67" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="36" customHeight="1">
-      <x:c r="A68" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B68" s="14" t="n">
-        <x:v>46229.26736111111</x:v>
-      </x:c>
-      <x:c r="C68" s="14" t="n">
-        <x:v>46229.29861111111</x:v>
-      </x:c>
-      <x:c r="D68" s="13" t="n">
-        <x:v>0.03125</x:v>
-      </x:c>
-      <x:c r="E68" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F68" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G68" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69" ht="36" customHeight="1">
-      <x:c r="A69" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B69" s="14" t="n">
-        <x:v>46229.305555555555</x:v>
-      </x:c>
-      <x:c r="C69" s="14" t="n">
-        <x:v>46229.3125</x:v>
-      </x:c>
-      <x:c r="D69" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E69" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F69" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G69" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="36" customHeight="1">
-      <x:c r="A70" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B70" s="14" t="n">
-        <x:v>46229.319444444445</x:v>
-      </x:c>
-      <x:c r="C70" s="14" t="n">
-        <x:v>46229.368055555555</x:v>
-      </x:c>
-      <x:c r="D70" s="13" t="n">
-        <x:v>0.0486111111</x:v>
-      </x:c>
-      <x:c r="E70" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F70" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G70" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="36" customHeight="1">
-      <x:c r="A71" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B71" s="14" t="n">
-        <x:v>46229.375</x:v>
-      </x:c>
-      <x:c r="C71" s="14" t="n">
-        <x:v>46229.38888888889</x:v>
-      </x:c>
-      <x:c r="D71" s="13" t="n">
-        <x:v>0.0138888889</x:v>
-      </x:c>
-      <x:c r="E71" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F71" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G71" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="36" customHeight="1">
-      <x:c r="A72" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B72" s="14" t="n">
-        <x:v>46229.39236111111</x:v>
-      </x:c>
-      <x:c r="C72" s="14" t="n">
-        <x:v>46229.395833333336</x:v>
-      </x:c>
-      <x:c r="D72" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E72" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F72" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G72" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="36" customHeight="1">
-      <x:c r="A73" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B73" s="14" t="n">
-        <x:v>46229.40277777778</x:v>
-      </x:c>
-      <x:c r="C73" s="14" t="n">
-        <x:v>46229.416666666664</x:v>
-      </x:c>
-      <x:c r="D73" s="13" t="n">
-        <x:v>0.0138888889</x:v>
-      </x:c>
-      <x:c r="E73" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F73" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G73" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="36" customHeight="1">
-      <x:c r="A74" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B74" s="14" t="n">
-        <x:v>46229.42361111111</x:v>
-      </x:c>
-      <x:c r="C74" s="14" t="n">
-        <x:v>46229.427083333336</x:v>
-      </x:c>
-      <x:c r="D74" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E74" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F74" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G74" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="36" customHeight="1">
-      <x:c r="A75" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B75" s="14" t="n">
-        <x:v>46229.43402777778</x:v>
-      </x:c>
-      <x:c r="C75" s="14" t="n">
-        <x:v>46229.444444444445</x:v>
-      </x:c>
-      <x:c r="D75" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E75" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F75" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G75" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76" ht="36" customHeight="1">
-      <x:c r="A76" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B76" s="14" t="n">
-        <x:v>46229.447916666664</x:v>
-      </x:c>
-      <x:c r="C76" s="14" t="n">
-        <x:v>46231.90972222222</x:v>
-      </x:c>
-      <x:c r="D76" s="13" t="n">
-        <x:v>2.4618055556</x:v>
-      </x:c>
-      <x:c r="E76" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F76" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G76" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="36" customHeight="1">
-      <x:c r="A77" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B77" s="14" t="n">
-        <x:v>46231.92361111111</x:v>
-      </x:c>
-      <x:c r="C77" s="14" t="n">
-        <x:v>46231.927083333336</x:v>
-      </x:c>
-      <x:c r="D77" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E77" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F77" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G77" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="36" customHeight="1">
-      <x:c r="A78" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B78" s="14" t="n">
-        <x:v>46231.930555555555</x:v>
-      </x:c>
-      <x:c r="C78" s="14" t="n">
-        <x:v>46231.93402777778</x:v>
-      </x:c>
-      <x:c r="D78" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E78" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F78" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G78" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="36" customHeight="1">
-      <x:c r="A79" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B79" s="14" t="n">
-        <x:v>46231.9375</x:v>
-      </x:c>
-      <x:c r="C79" s="14" t="n">
-        <x:v>46232.381944444445</x:v>
-      </x:c>
-      <x:c r="D79" s="13" t="n">
-        <x:v>0.4444444444</x:v>
-      </x:c>
-      <x:c r="E79" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F79" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G79" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="36" customHeight="1">
-      <x:c r="A80" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B80" s="14" t="n">
-        <x:v>46232.38888888889</x:v>
-      </x:c>
-      <x:c r="C80" s="14" t="n">
-        <x:v>46232.399305555555</x:v>
-      </x:c>
-      <x:c r="D80" s="13" t="n">
-        <x:v>0.0104166667</x:v>
-      </x:c>
-      <x:c r="E80" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F80" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G80" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="36" customHeight="1">
-      <x:c r="A81" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B81" s="14" t="n">
-        <x:v>46232.40625</x:v>
-      </x:c>
-      <x:c r="C81" s="14" t="n">
-        <x:v>46232.572916666664</x:v>
-      </x:c>
-      <x:c r="D81" s="13" t="n">
-        <x:v>0.1666666667</x:v>
-      </x:c>
-      <x:c r="E81" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F81" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G81" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="36" customHeight="1">
-      <x:c r="A82" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B82" s="14" t="n">
-        <x:v>46232.57638888889</x:v>
-      </x:c>
-      <x:c r="C82" s="14" t="n">
-        <x:v>46232.57986111111</x:v>
-      </x:c>
-      <x:c r="D82" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E82" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F82" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G82" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="36" customHeight="1">
-      <x:c r="A83" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B83" s="14" t="n">
-        <x:v>46232.59027777778</x:v>
-      </x:c>
-      <x:c r="C83" s="14" t="n">
-        <x:v>46232.59375</x:v>
-      </x:c>
-      <x:c r="D83" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E83" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F83" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G83" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84" ht="36" customHeight="1">
-      <x:c r="A84" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B84" s="14" t="n">
-        <x:v>46232.59722222222</x:v>
-      </x:c>
-      <x:c r="C84" s="14" t="n">
-        <x:v>46232.600694444445</x:v>
-      </x:c>
-      <x:c r="D84" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E84" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F84" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G84" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="36" customHeight="1">
-      <x:c r="A85" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B85" s="14" t="n">
-        <x:v>46232.60763888889</x:v>
-      </x:c>
-      <x:c r="C85" s="14" t="n">
-        <x:v>46232.649305555555</x:v>
-      </x:c>
-      <x:c r="D85" s="13" t="n">
-        <x:v>0.0416666667</x:v>
-      </x:c>
-      <x:c r="E85" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F85" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G85" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="36" customHeight="1">
-      <x:c r="A86" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B86" s="14" t="n">
-        <x:v>46232.65625</x:v>
-      </x:c>
-      <x:c r="C86" s="14" t="n">
-        <x:v>46232.663194444445</x:v>
-      </x:c>
-      <x:c r="D86" s="13" t="n">
-        <x:v>0.0069444444</x:v>
-      </x:c>
-      <x:c r="E86" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F86" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G86" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="36" customHeight="1">
-      <x:c r="A87" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B87" s="14" t="n">
-        <x:v>46232.67013888889</x:v>
-      </x:c>
-      <x:c r="C87" s="14" t="n">
-        <x:v>46232.694444444445</x:v>
-      </x:c>
-      <x:c r="D87" s="13" t="n">
-        <x:v>0.0243055556</x:v>
-      </x:c>
-      <x:c r="E87" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F87" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G87" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="36" customHeight="1">
-      <x:c r="A88" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B88" s="14" t="n">
-        <x:v>46232.70486111111</x:v>
-      </x:c>
-      <x:c r="C88" s="14" t="n">
-        <x:v>46232.708333333336</x:v>
-      </x:c>
-      <x:c r="D88" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E88" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F88" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G88" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="36" customHeight="1">
-      <x:c r="A89" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B89" s="14" t="n">
-        <x:v>46232.72222222222</x:v>
-      </x:c>
-      <x:c r="C89" s="14" t="n">
-        <x:v>46232.73611111111</x:v>
-      </x:c>
-      <x:c r="D89" s="13" t="n">
-        <x:v>0.0138888889</x:v>
-      </x:c>
-      <x:c r="E89" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F89" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G89" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="36" customHeight="1">
-      <x:c r="A90" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B90" s="14" t="n">
-        <x:v>46232.739583333336</x:v>
-      </x:c>
-      <x:c r="C90" s="14" t="n">
-        <x:v>46232.90625</x:v>
-      </x:c>
-      <x:c r="D90" s="13" t="n">
-        <x:v>0.1666666667</x:v>
-      </x:c>
-      <x:c r="E90" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F90" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G90" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="36" customHeight="1">
-      <x:c r="A91" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B91" s="14" t="n">
-        <x:v>46232.913194444445</x:v>
-      </x:c>
-      <x:c r="C91" s="14" t="n">
-        <x:v>46232.93402777778</x:v>
-      </x:c>
-      <x:c r="D91" s="13" t="n">
-        <x:v>0.0208333333</x:v>
-      </x:c>
-      <x:c r="E91" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F91" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G91" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="36" customHeight="1">
-      <x:c r="A92" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B92" s="14" t="n">
-        <x:v>46232.9375</x:v>
-      </x:c>
-      <x:c r="C92" s="14" t="n">
-        <x:v>46232.94097222222</x:v>
-      </x:c>
-      <x:c r="D92" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E92" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F92" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G92" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="36" customHeight="1">
-      <x:c r="A93" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B93" s="14" t="n">
-        <x:v>46232.947916666664</x:v>
-      </x:c>
-      <x:c r="C93" s="14" t="n">
-        <x:v>46233.913194444445</x:v>
-      </x:c>
-      <x:c r="D93" s="13" t="n">
-        <x:v>0.9652777778</x:v>
-      </x:c>
-      <x:c r="E93" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F93" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G93" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="36" customHeight="1">
-      <x:c r="A94" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B94" s="14" t="n">
-        <x:v>46233.927083333336</x:v>
-      </x:c>
-      <x:c r="C94" s="14" t="n">
-        <x:v>46233.930555555555</x:v>
-      </x:c>
-      <x:c r="D94" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E94" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F94" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G94" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95" ht="36" customHeight="1">
-      <x:c r="A95" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B95" s="14" t="n">
-        <x:v>46233.94097222222</x:v>
-      </x:c>
-      <x:c r="C95" s="14" t="n">
-        <x:v>46233.944444444445</x:v>
-      </x:c>
-      <x:c r="D95" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E95" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F95" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G95" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="36" customHeight="1">
-      <x:c r="A96" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B96" s="14" t="n">
-        <x:v>46233.95138888889</x:v>
-      </x:c>
-      <x:c r="C96" s="14" t="n">
-        <x:v>46233.97222222222</x:v>
-      </x:c>
-      <x:c r="D96" s="13" t="n">
-        <x:v>0.0208333333</x:v>
-      </x:c>
-      <x:c r="E96" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F96" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G96" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="36" customHeight="1">
-      <x:c r="A97" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B97" s="14" t="n">
-        <x:v>46233.979166666664</x:v>
-      </x:c>
-      <x:c r="C97" s="14" t="n">
-        <x:v>46233.98263888889</x:v>
-      </x:c>
-      <x:c r="D97" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E97" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F97" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G97" s="15" t="b">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98" ht="36" customHeight="1">
-      <x:c r="A98" s="13" t="str">
-        <x:v>Eight DO + 12 process inputs (units pending)</x:v>
-      </x:c>
-      <x:c r="B98" s="14" t="n">
-        <x:v>46233.99652777778</x:v>
-      </x:c>
-      <x:c r="C98" s="14" t="n">
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="D98" s="13" t="n">
-        <x:v>0.0034722222</x:v>
-      </x:c>
-      <x:c r="E98" s="13" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F98" s="13" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G98" s="15" t="b">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4265,10 +2770,10 @@
         <x:v>进水瞬时流量（m³/h）</x:v>
       </x:c>
       <x:c r="B2" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C2" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
@@ -4276,10 +2781,10 @@
         <x:v>出水瞬时流量（m³/h）</x:v>
       </x:c>
       <x:c r="B3" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C3" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.5561985597</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
@@ -4287,10 +2792,10 @@
         <x:v>进水pH</x:v>
       </x:c>
       <x:c r="B4" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C4" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
@@ -4298,10 +2803,10 @@
         <x:v>进水COD（mg/L）</x:v>
       </x:c>
       <x:c r="B5" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C5" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
@@ -4309,10 +2814,10 @@
         <x:v>进水氨氮（mg/L）</x:v>
       </x:c>
       <x:c r="B6" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C6" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
@@ -4320,10 +2825,10 @@
         <x:v>进水温度（℃）</x:v>
       </x:c>
       <x:c r="B7" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C7" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="22" customHeight="1">
@@ -4331,10 +2836,10 @@
         <x:v>进水总磷（mg/L）</x:v>
       </x:c>
       <x:c r="B8" s="7" t="n">
-        <x:v>140</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C8" s="6" t="n">
-        <x:v>0.4501028807</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -4342,10 +2847,10 @@
         <x:v>进水总氮（mg/L）</x:v>
       </x:c>
       <x:c r="B9" s="7" t="n">
-        <x:v>232</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C9" s="6" t="n">
-        <x:v>0.7458847737</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
@@ -4353,10 +2858,10 @@
         <x:v>进水SS（mg/L）</x:v>
       </x:c>
       <x:c r="B10" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="C10" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>1.5207047325</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
@@ -4364,10 +2869,10 @@
         <x:v>出水pH</x:v>
       </x:c>
       <x:c r="B11" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C11" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
@@ -4375,10 +2880,10 @@
         <x:v>出水COD（mg/L）</x:v>
       </x:c>
       <x:c r="B12" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C12" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
@@ -4386,10 +2891,10 @@
         <x:v>出水氨氮（mg/L）</x:v>
       </x:c>
       <x:c r="B13" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C13" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
@@ -4397,10 +2902,10 @@
         <x:v>出水温度（℃）</x:v>
       </x:c>
       <x:c r="B14" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C14" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
@@ -4408,10 +2913,10 @@
         <x:v>出水总磷（mg/L）</x:v>
       </x:c>
       <x:c r="B15" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C15" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
@@ -4419,10 +2924,10 @@
         <x:v>出水总氮（mg/L）</x:v>
       </x:c>
       <x:c r="B16" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C16" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
@@ -4430,10 +2935,10 @@
         <x:v>氯化铁流量计1（m³/h）</x:v>
       </x:c>
       <x:c r="B17" s="7" t="n">
-        <x:v>165</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C17" s="6" t="n">
-        <x:v>0.5304783951</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
@@ -4441,10 +2946,10 @@
         <x:v>氯化铁流量计2（m³/h）</x:v>
       </x:c>
       <x:c r="B18" s="7" t="n">
-        <x:v>1942</x:v>
+        <x:v>1928</x:v>
       </x:c>
       <x:c r="C18" s="6" t="n">
-        <x:v>6.2435699588</x:v>
+        <x:v>6.1985596708</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
@@ -4452,10 +2957,10 @@
         <x:v>乙酸钠流量计2（m³/h）</x:v>
       </x:c>
       <x:c r="B19" s="7" t="n">
-        <x:v>153</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C19" s="6" t="n">
-        <x:v>0.4918981481</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
@@ -4463,10 +2968,10 @@
         <x:v>乙酸钠流量计4（m³/h）</x:v>
       </x:c>
       <x:c r="B20" s="7" t="n">
-        <x:v>165</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C20" s="6" t="n">
-        <x:v>0.5304783951</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
@@ -4474,10 +2979,10 @@
         <x:v>FIT1531A排泥流量（m³/h）</x:v>
       </x:c>
       <x:c r="B21" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C21" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
@@ -4485,10 +2990,10 @@
         <x:v>FIT1531B排泥流量（m³/h）</x:v>
       </x:c>
       <x:c r="B22" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C22" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
@@ -4496,10 +3001,10 @@
         <x:v>1#生物池外回流流量（m³/h）</x:v>
       </x:c>
       <x:c r="B23" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C23" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
@@ -4507,10 +3012,10 @@
         <x:v>2#生物池外回流流量（m³/h）</x:v>
       </x:c>
       <x:c r="B24" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C24" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
@@ -4518,10 +3023,10 @@
         <x:v>1#生物池内回流流量（m³/h）</x:v>
       </x:c>
       <x:c r="B25" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C25" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
@@ -4529,10 +3034,10 @@
         <x:v>2#生物池内回流流量（m³/h）</x:v>
       </x:c>
       <x:c r="B26" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C26" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
@@ -4540,10 +3045,10 @@
         <x:v>剩余污泥流量（m³/h）</x:v>
       </x:c>
       <x:c r="B27" s="7" t="n">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C27" s="6" t="n">
-        <x:v>0.1221707819</x:v>
+        <x:v>0.0964506173</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
@@ -4562,10 +3067,10 @@
         <x:v>进水瞬时流量（m³/d）</x:v>
       </x:c>
       <x:c r="B29" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C29" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
@@ -4573,10 +3078,10 @@
         <x:v>出水瞬时流量（m³/d）</x:v>
       </x:c>
       <x:c r="B30" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="C30" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.5561985597</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
@@ -4584,10 +3089,10 @@
         <x:v>氯化铁流量计1（m³/d）</x:v>
       </x:c>
       <x:c r="B31" s="7" t="n">
-        <x:v>165</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C31" s="6" t="n">
-        <x:v>0.5304783951</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
@@ -4595,10 +3100,10 @@
         <x:v>氯化铁流量计2（m³/d）</x:v>
       </x:c>
       <x:c r="B32" s="7" t="n">
-        <x:v>1942</x:v>
+        <x:v>1928</x:v>
       </x:c>
       <x:c r="C32" s="6" t="n">
-        <x:v>6.2435699588</x:v>
+        <x:v>6.1985596708</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
@@ -4606,10 +3111,10 @@
         <x:v>乙酸钠流量计2（m³/d）</x:v>
       </x:c>
       <x:c r="B33" s="7" t="n">
-        <x:v>153</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C33" s="6" t="n">
-        <x:v>0.4918981481</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
@@ -4617,10 +3122,10 @@
         <x:v>乙酸钠流量计4（m³/d）</x:v>
       </x:c>
       <x:c r="B34" s="7" t="n">
-        <x:v>165</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="C34" s="6" t="n">
-        <x:v>0.5304783951</x:v>
+        <x:v>0.4726080247</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="22" customHeight="1">
@@ -4628,10 +3133,10 @@
         <x:v>FIT1531A排泥流量（m³/d）</x:v>
       </x:c>
       <x:c r="B35" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C35" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="22" customHeight="1">
@@ -4639,10 +3144,10 @@
         <x:v>FIT1531B排泥流量（m³/d）</x:v>
       </x:c>
       <x:c r="B36" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C36" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="22" customHeight="1">
@@ -4650,10 +3155,10 @@
         <x:v>1#生物池外回流流量（m³/d）</x:v>
       </x:c>
       <x:c r="B37" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C37" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="22" customHeight="1">
@@ -4661,10 +3166,10 @@
         <x:v>2#生物池外回流流量（m³/d）</x:v>
       </x:c>
       <x:c r="B38" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C38" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
@@ -4672,10 +3177,10 @@
         <x:v>1#生物池内回流流量（m³/d）</x:v>
       </x:c>
       <x:c r="B39" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C39" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="22" customHeight="1">
@@ -4683,10 +3188,10 @@
         <x:v>2#生物池内回流流量（m³/d）</x:v>
       </x:c>
       <x:c r="B40" s="7" t="n">
-        <x:v>118</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C40" s="6" t="n">
-        <x:v>0.379372428</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
@@ -4694,10 +3199,10 @@
         <x:v>剩余污泥流量（m³/d）</x:v>
       </x:c>
       <x:c r="B41" s="7" t="n">
-        <x:v>38</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C41" s="6" t="n">
-        <x:v>0.1221707819</x:v>
+        <x:v>0.0964506173</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="22" customHeight="1">
@@ -4705,10 +3210,10 @@
         <x:v>MBR循环流（m³/d）</x:v>
       </x:c>
       <x:c r="B42" s="7" t="n">
-        <x:v>156</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="C42" s="6" t="n">
-        <x:v>0.5015432099</x:v>
+        <x:v>0.4565329218</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="22" customHeight="1">
@@ -4716,10 +3221,10 @@
         <x:v>frSNHx_TKN（氨氮/总氮）</x:v>
       </x:c>
       <x:c r="B43" s="7" t="n">
-        <x:v>235</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="C43" s="6" t="n">
-        <x:v>0.7555298354</x:v>
+        <x:v>0.3600823045</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="22" customHeight="1">
@@ -4727,10 +3232,10 @@
         <x:v>frSU_SCCOD代理量（mg/L）</x:v>
       </x:c>
       <x:c r="B44" s="7" t="n">
-        <x:v>151</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C44" s="6" t="n">
-        <x:v>0.485468107</x:v>
+        <x:v>0.2700617284</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4919,7 +3424,7 @@
         <x:v>Selected pilot: start</x:v>
       </x:c>
       <x:c r="B22" s="13" t="str">
-        <x:v>2026-04-10 00:00:00</x:v>
+        <x:v>2026-03-31 00:00:00</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="32" customHeight="1">
@@ -4927,7 +3432,7 @@
         <x:v>Selected pilot: end exclusive</x:v>
       </x:c>
       <x:c r="B23" s="13" t="str">
-        <x:v>2026-05-08 00:00:00</x:v>
+        <x:v>2026-04-28 00:00:00</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="32" customHeight="1">
@@ -4935,7 +3440,7 @@
         <x:v>Selected pilot: evaluation start</x:v>
       </x:c>
       <x:c r="B24" s="13" t="str">
-        <x:v>2026-04-24 00:00:00</x:v>
+        <x:v>2026-04-14 00:00:00</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="32" customHeight="1">

</xml_diff>